<commit_message>
Price each agent's savings at its role's BLS median pay
Replace the flat $40/hour with the median pay (BLS, May 2025) of the role
that would normally do each job, plus benefits. Updates the book, the
savings calculator and the /agents page copy.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VC6mEVfjHSo5id2svPT1oA
</commit_message>
<xml_diff>
--- a/files/agent-savings-calculator.xlsx
+++ b/files/agent-savings-calculator.xlsx
@@ -96,11 +96,11 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -470,20 +470,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:M36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,14 +502,11 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Your hourly cost ($)</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>40</v>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Default hourly cost = the role's BLS median pay (May 2025) ÷ 0.70 for benefits and payroll taxes. Replace it with what you actually pay.</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -538,40 +537,50 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
+          <t>Who would do it by hand</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Hourly cost ($)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>Minutes by hand (per run)</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Minutes to review (per run)</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Runs per month</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Hours saved / month</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Time savings / month</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Direct savings / month ($)</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
         <is>
           <t>Building it? (Y/N)</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>Counted savings / month</t>
         </is>
@@ -591,33 +600,41 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Executive assistant</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F8" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="G8" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="H8" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="G8" s="9">
-        <f>MAX(0,(D8-E8)*F8/60)</f>
-        <v/>
-      </c>
-      <c r="H8" s="10">
-        <f>G8*$C$4</f>
-        <v/>
-      </c>
-      <c r="I8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K8" s="10">
-        <f>IF(UPPER(J8)="Y",H8+I8,0)</f>
+      <c r="I8" s="10">
+        <f>MAX(0,(F8-G8)*H8/60)</f>
+        <v/>
+      </c>
+      <c r="J8" s="11">
+        <f>I8*E8</f>
+        <v/>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M8" s="11">
+        <f>IF(UPPER(L8)="Y",J8+K8,0)</f>
         <v/>
       </c>
     </row>
@@ -635,33 +652,41 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Executive assistant</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F9" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="G9" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="H9" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="G9" s="9">
-        <f>MAX(0,(D9-E9)*F9/60)</f>
-        <v/>
-      </c>
-      <c r="H9" s="10">
-        <f>G9*$C$4</f>
-        <v/>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K9" s="10">
-        <f>IF(UPPER(J9)="Y",H9+I9,0)</f>
+      <c r="I9" s="10">
+        <f>MAX(0,(F9-G9)*H9/60)</f>
+        <v/>
+      </c>
+      <c r="J9" s="11">
+        <f>I9*E9</f>
+        <v/>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M9" s="11">
+        <f>IF(UPPER(L9)="Y",J9+K9,0)</f>
         <v/>
       </c>
     </row>
@@ -679,33 +704,41 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Technical writer</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="F10" s="8" t="n">
         <v>240</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="G10" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F10" s="8" t="n">
+      <c r="H10" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="9">
-        <f>MAX(0,(D10-E10)*F10/60)</f>
-        <v/>
-      </c>
-      <c r="H10" s="10">
-        <f>G10*$C$4</f>
-        <v/>
-      </c>
-      <c r="I10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K10" s="10">
-        <f>IF(UPPER(J10)="Y",H10+I10,0)</f>
+      <c r="I10" s="10">
+        <f>MAX(0,(F10-G10)*H10/60)</f>
+        <v/>
+      </c>
+      <c r="J10" s="11">
+        <f>I10*E10</f>
+        <v/>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M10" s="11">
+        <f>IF(UPPER(L10)="Y",J10+K10,0)</f>
         <v/>
       </c>
     </row>
@@ -723,33 +756,41 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Management analyst</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="F11" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="G11" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="H11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="9">
-        <f>MAX(0,(D11-E11)*F11/60)</f>
-        <v/>
-      </c>
-      <c r="H11" s="10">
-        <f>G11*$C$4</f>
-        <v/>
-      </c>
-      <c r="I11" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K11" s="10">
-        <f>IF(UPPER(J11)="Y",H11+I11,0)</f>
+      <c r="I11" s="10">
+        <f>MAX(0,(F11-G11)*H11/60)</f>
+        <v/>
+      </c>
+      <c r="J11" s="11">
+        <f>I11*E11</f>
+        <v/>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M11" s="11">
+        <f>IF(UPPER(L11)="Y",J11+K11,0)</f>
         <v/>
       </c>
     </row>
@@ -767,33 +808,41 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n">
-        <v>20</v>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Sales representative</t>
+        </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="F12" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="G12" s="9">
-        <f>MAX(0,(D12-E12)*F12/60)</f>
-        <v/>
-      </c>
-      <c r="H12" s="10">
-        <f>G12*$C$4</f>
-        <v/>
-      </c>
-      <c r="I12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K12" s="10">
-        <f>IF(UPPER(J12)="Y",H12+I12,0)</f>
+      <c r="G12" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" s="10">
+        <f>MAX(0,(F12-G12)*H12/60)</f>
+        <v/>
+      </c>
+      <c r="J12" s="11">
+        <f>I12*E12</f>
+        <v/>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M12" s="11">
+        <f>IF(UPPER(L12)="Y",J12+K12,0)</f>
         <v/>
       </c>
     </row>
@@ -811,33 +860,41 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Sales representative</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F13" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="G13" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="H13" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="G13" s="9">
-        <f>MAX(0,(D13-E13)*F13/60)</f>
-        <v/>
-      </c>
-      <c r="H13" s="10">
-        <f>G13*$C$4</f>
-        <v/>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K13" s="10">
-        <f>IF(UPPER(J13)="Y",H13+I13,0)</f>
+      <c r="I13" s="10">
+        <f>MAX(0,(F13-G13)*H13/60)</f>
+        <v/>
+      </c>
+      <c r="J13" s="11">
+        <f>I13*E13</f>
+        <v/>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M13" s="11">
+        <f>IF(UPPER(L13)="Y",J13+K13,0)</f>
         <v/>
       </c>
     </row>
@@ -855,33 +912,41 @@
           <t>Sales</t>
         </is>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Sales representative</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="G14" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="H14" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G14" s="9">
-        <f>MAX(0,(D14-E14)*F14/60)</f>
-        <v/>
-      </c>
-      <c r="H14" s="10">
-        <f>G14*$C$4</f>
-        <v/>
-      </c>
-      <c r="I14" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K14" s="10">
-        <f>IF(UPPER(J14)="Y",H14+I14,0)</f>
+      <c r="I14" s="10">
+        <f>MAX(0,(F14-G14)*H14/60)</f>
+        <v/>
+      </c>
+      <c r="J14" s="11">
+        <f>I14*E14</f>
+        <v/>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M14" s="11">
+        <f>IF(UPPER(L14)="Y",J14+K14,0)</f>
         <v/>
       </c>
     </row>
@@ -899,33 +964,41 @@
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Marketing specialist</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="F15" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="G15" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="H15" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="9">
-        <f>MAX(0,(D15-E15)*F15/60)</f>
-        <v/>
-      </c>
-      <c r="H15" s="10">
-        <f>G15*$C$4</f>
-        <v/>
-      </c>
-      <c r="I15" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K15" s="10">
-        <f>IF(UPPER(J15)="Y",H15+I15,0)</f>
+      <c r="I15" s="10">
+        <f>MAX(0,(F15-G15)*H15/60)</f>
+        <v/>
+      </c>
+      <c r="J15" s="11">
+        <f>I15*E15</f>
+        <v/>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M15" s="11">
+        <f>IF(UPPER(L15)="Y",J15+K15,0)</f>
         <v/>
       </c>
     </row>
@@ -943,33 +1016,41 @@
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Writer</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="G16" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F16" s="8" t="n">
+      <c r="H16" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G16" s="9">
-        <f>MAX(0,(D16-E16)*F16/60)</f>
-        <v/>
-      </c>
-      <c r="H16" s="10">
-        <f>G16*$C$4</f>
-        <v/>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K16" s="10">
-        <f>IF(UPPER(J16)="Y",H16+I16,0)</f>
+      <c r="I16" s="10">
+        <f>MAX(0,(F16-G16)*H16/60)</f>
+        <v/>
+      </c>
+      <c r="J16" s="11">
+        <f>I16*E16</f>
+        <v/>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M16" s="11">
+        <f>IF(UPPER(L16)="Y",J16+K16,0)</f>
         <v/>
       </c>
     </row>
@@ -987,33 +1068,41 @@
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Market research analyst</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="F17" s="8" t="n">
         <v>240</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="G17" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="H17" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="9">
-        <f>MAX(0,(D17-E17)*F17/60)</f>
-        <v/>
-      </c>
-      <c r="H17" s="10">
-        <f>G17*$C$4</f>
-        <v/>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K17" s="10">
-        <f>IF(UPPER(J17)="Y",H17+I17,0)</f>
+      <c r="I17" s="10">
+        <f>MAX(0,(F17-G17)*H17/60)</f>
+        <v/>
+      </c>
+      <c r="J17" s="11">
+        <f>I17*E17</f>
+        <v/>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M17" s="11">
+        <f>IF(UPPER(L17)="Y",J17+K17,0)</f>
         <v/>
       </c>
     </row>
@@ -1031,33 +1120,41 @@
           <t>Marketing</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Customer service rep</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="F18" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="E18" s="7" t="n">
+      <c r="G18" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F18" s="8" t="n">
+      <c r="H18" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="G18" s="9">
-        <f>MAX(0,(D18-E18)*F18/60)</f>
-        <v/>
-      </c>
-      <c r="H18" s="10">
-        <f>G18*$C$4</f>
-        <v/>
-      </c>
-      <c r="I18" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K18" s="10">
-        <f>IF(UPPER(J18)="Y",H18+I18,0)</f>
+      <c r="I18" s="10">
+        <f>MAX(0,(F18-G18)*H18/60)</f>
+        <v/>
+      </c>
+      <c r="J18" s="11">
+        <f>I18*E18</f>
+        <v/>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M18" s="11">
+        <f>IF(UPPER(L18)="Y",J18+K18,0)</f>
         <v/>
       </c>
     </row>
@@ -1075,33 +1172,41 @@
           <t>Customer service</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Customer service rep</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="F19" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E19" s="7" t="n">
+      <c r="G19" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="H19" s="9" t="n">
         <v>96</v>
       </c>
-      <c r="G19" s="9">
-        <f>MAX(0,(D19-E19)*F19/60)</f>
-        <v/>
-      </c>
-      <c r="H19" s="10">
-        <f>G19*$C$4</f>
-        <v/>
-      </c>
-      <c r="I19" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K19" s="10">
-        <f>IF(UPPER(J19)="Y",H19+I19,0)</f>
+      <c r="I19" s="10">
+        <f>MAX(0,(F19-G19)*H19/60)</f>
+        <v/>
+      </c>
+      <c r="J19" s="11">
+        <f>I19*E19</f>
+        <v/>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M19" s="11">
+        <f>IF(UPPER(L19)="Y",J19+K19,0)</f>
         <v/>
       </c>
     </row>
@@ -1119,33 +1224,41 @@
           <t>Customer service</t>
         </is>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Market research analyst</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>240</v>
       </c>
-      <c r="E20" s="7" t="n">
+      <c r="G20" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F20" s="8" t="n">
+      <c r="H20" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="9">
-        <f>MAX(0,(D20-E20)*F20/60)</f>
-        <v/>
-      </c>
-      <c r="H20" s="10">
-        <f>G20*$C$4</f>
-        <v/>
-      </c>
-      <c r="I20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K20" s="10">
-        <f>IF(UPPER(J20)="Y",H20+I20,0)</f>
+      <c r="I20" s="10">
+        <f>MAX(0,(F20-G20)*H20/60)</f>
+        <v/>
+      </c>
+      <c r="J20" s="11">
+        <f>I20*E20</f>
+        <v/>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M20" s="11">
+        <f>IF(UPPER(L20)="Y",J20+K20,0)</f>
         <v/>
       </c>
     </row>
@@ -1163,33 +1276,41 @@
           <t>Customer service</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Customer service rep</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="F21" s="8" t="n">
         <v>120</v>
       </c>
-      <c r="E21" s="7" t="n">
+      <c r="G21" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="H21" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="9">
-        <f>MAX(0,(D21-E21)*F21/60)</f>
-        <v/>
-      </c>
-      <c r="H21" s="10">
-        <f>G21*$C$4</f>
-        <v/>
-      </c>
-      <c r="I21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K21" s="10">
-        <f>IF(UPPER(J21)="Y",H21+I21,0)</f>
+      <c r="I21" s="10">
+        <f>MAX(0,(F21-G21)*H21/60)</f>
+        <v/>
+      </c>
+      <c r="J21" s="11">
+        <f>I21*E21</f>
+        <v/>
+      </c>
+      <c r="K21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M21" s="11">
+        <f>IF(UPPER(L21)="Y",J21+K21,0)</f>
         <v/>
       </c>
     </row>
@@ -1207,33 +1328,41 @@
           <t>Finance</t>
         </is>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Bill and account collector</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="F22" s="8" t="n">
         <v>240</v>
       </c>
-      <c r="E22" s="7" t="n">
+      <c r="G22" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="H22" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="9">
-        <f>MAX(0,(D22-E22)*F22/60)</f>
-        <v/>
-      </c>
-      <c r="H22" s="10">
-        <f>G22*$C$4</f>
-        <v/>
-      </c>
-      <c r="I22" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K22" s="10">
-        <f>IF(UPPER(J22)="Y",H22+I22,0)</f>
+      <c r="I22" s="10">
+        <f>MAX(0,(F22-G22)*H22/60)</f>
+        <v/>
+      </c>
+      <c r="J22" s="11">
+        <f>I22*E22</f>
+        <v/>
+      </c>
+      <c r="K22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M22" s="11">
+        <f>IF(UPPER(L22)="Y",J22+K22,0)</f>
         <v/>
       </c>
     </row>
@@ -1251,33 +1380,41 @@
           <t>Finance</t>
         </is>
       </c>
-      <c r="D23" s="7" t="n">
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Bookkeeping clerk</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="F23" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="E23" s="7" t="n">
+      <c r="G23" s="8" t="n">
         <v>90</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="H23" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="9">
-        <f>MAX(0,(D23-E23)*F23/60)</f>
-        <v/>
-      </c>
-      <c r="H23" s="10">
-        <f>G23*$C$4</f>
-        <v/>
-      </c>
-      <c r="I23" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K23" s="10">
-        <f>IF(UPPER(J23)="Y",H23+I23,0)</f>
+      <c r="I23" s="10">
+        <f>MAX(0,(F23-G23)*H23/60)</f>
+        <v/>
+      </c>
+      <c r="J23" s="11">
+        <f>I23*E23</f>
+        <v/>
+      </c>
+      <c r="K23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M23" s="11">
+        <f>IF(UPPER(L23)="Y",J23+K23,0)</f>
         <v/>
       </c>
     </row>
@@ -1295,33 +1432,41 @@
           <t>Finance</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Accountant</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>57</v>
+      </c>
+      <c r="F24" s="8" t="n">
         <v>240</v>
       </c>
-      <c r="E24" s="7" t="n">
+      <c r="G24" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F24" s="8" t="n">
+      <c r="H24" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="9">
-        <f>MAX(0,(D24-E24)*F24/60)</f>
-        <v/>
-      </c>
-      <c r="H24" s="10">
-        <f>G24*$C$4</f>
-        <v/>
-      </c>
-      <c r="I24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K24" s="10">
-        <f>IF(UPPER(J24)="Y",H24+I24,0)</f>
+      <c r="I24" s="10">
+        <f>MAX(0,(F24-G24)*H24/60)</f>
+        <v/>
+      </c>
+      <c r="J24" s="11">
+        <f>I24*E24</f>
+        <v/>
+      </c>
+      <c r="K24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M24" s="11">
+        <f>IF(UPPER(L24)="Y",J24+K24,0)</f>
         <v/>
       </c>
     </row>
@@ -1339,34 +1484,42 @@
           <t>Finance</t>
         </is>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Bookkeeping clerk</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="F25" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E25" s="7" t="n">
+      <c r="G25" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="F25" s="8">
+      <c r="H25" s="9">
         <f>1/3</f>
         <v/>
       </c>
-      <c r="G25" s="9">
-        <f>MAX(0,(D25-E25)*F25/60)</f>
-        <v/>
-      </c>
-      <c r="H25" s="10">
-        <f>G25*$C$4</f>
-        <v/>
-      </c>
-      <c r="I25" s="11" t="n">
+      <c r="I25" s="10">
+        <f>MAX(0,(F25-G25)*H25/60)</f>
+        <v/>
+      </c>
+      <c r="J25" s="11">
+        <f>I25*E25</f>
+        <v/>
+      </c>
+      <c r="K25" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K25" s="10">
-        <f>IF(UPPER(J25)="Y",H25+I25,0)</f>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M25" s="11">
+        <f>IF(UPPER(L25)="Y",J25+K25,0)</f>
         <v/>
       </c>
     </row>
@@ -1384,34 +1537,42 @@
           <t>People</t>
         </is>
       </c>
-      <c r="D26" s="7" t="n">
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>HR specialist</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="F26" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="E26" s="7" t="n">
+      <c r="G26" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="F26" s="8">
+      <c r="H26" s="9">
         <f>1/3</f>
         <v/>
       </c>
-      <c r="G26" s="9">
-        <f>MAX(0,(D26-E26)*F26/60)</f>
-        <v/>
-      </c>
-      <c r="H26" s="10">
-        <f>G26*$C$4</f>
-        <v/>
-      </c>
-      <c r="I26" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K26" s="10">
-        <f>IF(UPPER(J26)="Y",H26+I26,0)</f>
+      <c r="I26" s="10">
+        <f>MAX(0,(F26-G26)*H26/60)</f>
+        <v/>
+      </c>
+      <c r="J26" s="11">
+        <f>I26*E26</f>
+        <v/>
+      </c>
+      <c r="K26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M26" s="11">
+        <f>IF(UPPER(L26)="Y",J26+K26,0)</f>
         <v/>
       </c>
     </row>
@@ -1429,33 +1590,41 @@
           <t>People</t>
         </is>
       </c>
-      <c r="D27" s="7" t="n">
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Operations manager</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>73</v>
+      </c>
+      <c r="F27" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="E27" s="7" t="n">
+      <c r="G27" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="F27" s="8" t="n">
+      <c r="H27" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G27" s="9">
-        <f>MAX(0,(D27-E27)*F27/60)</f>
-        <v/>
-      </c>
-      <c r="H27" s="10">
-        <f>G27*$C$4</f>
-        <v/>
-      </c>
-      <c r="I27" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K27" s="10">
-        <f>IF(UPPER(J27)="Y",H27+I27,0)</f>
+      <c r="I27" s="10">
+        <f>MAX(0,(F27-G27)*H27/60)</f>
+        <v/>
+      </c>
+      <c r="J27" s="11">
+        <f>I27*E27</f>
+        <v/>
+      </c>
+      <c r="K27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M27" s="11">
+        <f>IF(UPPER(L27)="Y",J27+K27,0)</f>
         <v/>
       </c>
     </row>
@@ -1465,12 +1634,12 @@
           <t>Total (agents marked Y)</t>
         </is>
       </c>
-      <c r="G28" s="12">
-        <f>SUMPRODUCT((UPPER(J8:J27)="Y")*G8:G27)</f>
-        <v/>
-      </c>
-      <c r="K28" s="13">
-        <f>SUM(K8:K27)</f>
+      <c r="I28" s="12">
+        <f>SUMPRODUCT((UPPER(L8:L27)="Y")*I8:I27)</f>
+        <v/>
+      </c>
+      <c r="M28" s="13">
+        <f>SUM(M8:M27)</f>
         <v/>
       </c>
     </row>
@@ -1481,7 +1650,7 @@
         </is>
       </c>
       <c r="C30" s="14">
-        <f>K28</f>
+        <f>M28</f>
         <v/>
       </c>
     </row>
@@ -1503,7 +1672,7 @@
         </is>
       </c>
       <c r="C32" s="14">
-        <f>K28-C5</f>
+        <f>M28-C5</f>
         <v/>
       </c>
     </row>
@@ -1514,7 +1683,7 @@
         </is>
       </c>
       <c r="C33" s="14">
-        <f>(K28-C5)*12</f>
+        <f>(M28-C5)*12</f>
         <v/>
       </c>
     </row>
@@ -1525,7 +1694,7 @@
         </is>
       </c>
       <c r="C34" s="15">
-        <f>IF(C5&gt;0,K28/C5,"")</f>
+        <f>IF(C5&gt;0,M28/C5,"")</f>
         <v/>
       </c>
     </row>
@@ -1538,7 +1707,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J8:J27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L8:L27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>